<commit_message>
Update Novartis test case file
</commit_message>
<xml_diff>
--- a/Excel test case Novartis Pharma Services AG .xlsx
+++ b/Excel test case Novartis Pharma Services AG .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Desktop\Final project\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD050DC-6511-48F0-9883-8A426D145AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A96405F7-663D-43E5-AA1C-3C7CABFA7A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="18">
   <si>
     <t>Внутри сети</t>
   </si>
@@ -127,9 +127,6 @@
   </si>
   <si>
     <t>На городской, Другое</t>
-  </si>
-  <si>
-    <t>2705</t>
   </si>
 </sst>
 </file>
@@ -1464,12 +1461,13 @@
         <f>IF(F21="Правильный ответ","Укажите продолжительность разговоров на тарифном плане, на котором сидит абонент 77010000055","")</f>
         <v>Укажите продолжительность разговоров на тарифном плане, на котором сидит абонент 77010000055</v>
       </c>
-      <c r="D22" s="37" t="s">
-        <v>18</v>
+      <c r="D22" s="37">
+        <f>SUMIF('База данных'!B:B, VLOOKUP(77010000055, 'База данных'!A:B, 2, 0), 'База данных'!E:E)</f>
+        <v>2705</v>
       </c>
       <c r="F22" s="11" t="str">
         <f t="shared" si="0"/>
-        <v>Неправильный ответ</v>
+        <v>Правильный ответ</v>
       </c>
       <c r="O22" s="5">
         <v>2705</v>
@@ -1480,13 +1478,13 @@
       <c r="A23" s="5">
         <v>21</v>
       </c>
-      <c r="B23" s="11" t="str">
+      <c r="B23" s="11">
         <f t="shared" si="1"/>
-        <v/>
+        <v>21</v>
       </c>
       <c r="C23" s="12" t="str">
         <f>IF(F22="Правильный ответ","Укажите абонента, у которого наибольшее начисление","")</f>
-        <v/>
+        <v>Укажите абонента, у которого наибольшее начисление</v>
       </c>
       <c r="D23" s="2">
         <f>_xlfn.XLOOKUP(MAX('База данных'!D:D),'База данных'!D:D,'База данных'!A:A)</f>

</xml_diff>